<commit_message>
Add advanced cancel booking flow with queue recalculation
</commit_message>
<xml_diff>
--- a/backend/users.xlsx
+++ b/backend/users.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -621,14 +621,114 @@
           <t>zainab@gmail.com</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" t="n">
+        <v>1234567890</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>zainab123</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>sheerin</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>sheerin@gmail.com</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1234567890</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>sheerin12</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>hassain</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>hassain@gmail.com</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>7397280782</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>faazil12</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>banu</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>banu@gmail.com</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1234567890</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>banu12</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>hari</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>hari@gmail.com</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1234567890</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>hari12</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>afkhar</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>afkhar@gmail.com</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
         <is>
           <t>1234567890</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>zainab123</t>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>afkhar12</t>
         </is>
       </c>
     </row>

</xml_diff>